<commit_message>
Portal PO upload: a product only needs an identifier and a quantity
Rows with a supplier/client reference but no name (e.g. the HONGLI and
OGAZER sheets) were blocked as errors. The required rule is now: name OR
supplier ref OR client ref, plus quantity > 0. Template instructions
updated to match.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-pedido.xlsx
+++ b/public/templates/plantilla-pedido.xlsx
@@ -7584,7 +7584,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Llena la hoja «Pedido»: una fila por producto. No cambies los títulos de las columnas ni borres columnas. Luego sube el archivo en el portal, sección «Subir pedido».</t>
+          <t>Llena la hoja «Pedido»: una fila por producto. No cambies los títulos de las columnas ni borres columnas. Lo único obligatorio es identificar el producto (nombre o referencia) y la CANTIDAD. Luego sube el archivo en el portal, sección «Subir pedido».</t>
         </is>
       </c>
     </row>
@@ -7631,12 +7631,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>NOMBRE *</t>
+          <t>NOMBRE</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Nombre o descripción del producto. Obligatorio.</t>
+          <t>Nombre o descripción del producto. Obligatorio que el producto se pueda identificar: pon el NOMBRE, o la REF PROVEEDOR, o la REF CLIENTE (al menos una de las tres).</t>
         </is>
       </c>
     </row>

</xml_diff>